<commit_message>
contentBoard update / Kompetenzraster.xlsx added contentNodes Lvl 1-3
- Question Progress from DB
- Content-Node Level from DB
- Content Nodes Level 1-3, if content available (Kompetenzraster.xlsx)
</commit_message>
<xml_diff>
--- a/files/freetext_questions.xlsx
+++ b/files/freetext_questions.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcsauer/GitHub/hefl/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C68749-1DE0-AD4B-9876-11D449DF2DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BDE9B5A-0BCA-9C4D-9973-F6DFC62BCAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 

</xml_diff>

<commit_message>
Updated and added FreeText questions
o revised existing freetext questions (more points, more detailed expectations, grammar)
+ added some new questions

!! important
Question "Code: Rekursion" and "Code: Map" could be unsolvable, because the code snippets are not inside the question text itself.
</commit_message>
<xml_diff>
--- a/files/freetext_questions.xlsx
+++ b/files/freetext_questions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcsauer/GitHub/hefl/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jan\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BDE9B5A-0BCA-9C4D-9973-F6DFC62BCAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226ACC4B-B604-46CC-90BD-965543519A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t>Beschreibung</t>
   </si>
@@ -40,9 +40,6 @@
     <t>Definition Strings</t>
   </si>
   <si>
-    <t xml:space="preserve">Was sind Strings? Beschreibe Strings in eigenen Worten und gebe eine kurze Definition (1-2 Saetze) </t>
-  </si>
-  <si>
     <t>Definition: Was ist ein String</t>
   </si>
   <si>
@@ -52,9 +49,6 @@
     <t>Beispiel Strings</t>
   </si>
   <si>
-    <t>Gib ein Beispiel fuer einen String. Wie macht man einen String im Programmcode kenntlich.</t>
-  </si>
-  <si>
     <t>Beispiel: Angabe eines Beispiel-Strings</t>
   </si>
   <si>
@@ -67,18 +61,12 @@
     <t>Welche Operationen kann man auf strings anwenden? Nenne mindestens zwei.</t>
   </si>
   <si>
-    <t>Operationen: Nenne zwei Operationen die man auf strings anwenden kann</t>
-  </si>
-  <si>
     <t>Strings koennen mit + konkateniert und mit * und einer Zahl vervielfacht werden</t>
   </si>
   <si>
     <t>Methoden Strings</t>
   </si>
   <si>
-    <t>Welche Methoden gibt es fuer strings in python? Nenne mindestens zwei.</t>
-  </si>
-  <si>
     <t>Methoden: Nenne mindestens zwei Methoden von strings.</t>
   </si>
   <si>
@@ -100,9 +88,6 @@
     <t>Vorteile Rekursion</t>
   </si>
   <si>
-    <t>Welchen Vorteil von Rekursion haben wir kennengelernt? Nenne einen Vorteil aus der Vorlesung</t>
-  </si>
-  <si>
     <t>Vorteil: Nenne einen Vorteil von Rekursion aus der Vorlesung</t>
   </si>
   <si>
@@ -112,9 +97,6 @@
     <t>Definition Tupel</t>
   </si>
   <si>
-    <t>Was ist ein Tupel? Gib eine kurze Definition</t>
-  </si>
-  <si>
     <t>Definition: Gib eine kurze Definition von Tupeln</t>
   </si>
   <si>
@@ -124,9 +106,6 @@
     <t>Syntax Tupel</t>
   </si>
   <si>
-    <t>Wie definiert man ein Tupel? Schreibe ein Tupel mit den Elementen 3, 7 und 5 auf. (In dieser Reihenfolge)</t>
-  </si>
-  <si>
     <t>Syntax: Definiere das gegebene Tupel</t>
   </si>
   <si>
@@ -148,45 +127,21 @@
     <t>Beispiele mutable/immutable</t>
   </si>
   <si>
-    <t>Nenne jeweils zwei Beispiele fuer mutable/immutable Variablen in Python</t>
-  </si>
-  <si>
-    <t>Beispiele: Nenne jeweils zwei Beispiele fuer mutable/immutable Variablen</t>
-  </si>
-  <si>
     <t>Listen und Dictionaries sind mutable und strings und integer sind immutable</t>
   </si>
   <si>
     <t>Definition while loop</t>
   </si>
   <si>
-    <t>Wie funktioniert ein for loop? Gib eine kurze Definition in eigenen Worten</t>
-  </si>
-  <si>
-    <t>Definition: Wie funktioniert ein while loop</t>
-  </si>
-  <si>
-    <t>Ein while loop bekommt eine boolsche Bedingung die wiederholt geprueft werden kann. Solange diese Bedingung den Wert war hat wird ein Code Block ausgefuehrt bevor die Bedingung erneut geprueft wird.</t>
-  </si>
-  <si>
     <t>Definition Liste</t>
   </si>
   <si>
-    <t>Was ist eine Liste? Gib eine kurze Definition in eigenen Worten.</t>
-  </si>
-  <si>
-    <t>Definition: Was ist eine Liste</t>
-  </si>
-  <si>
     <t>Eine Liste ist eine Datenstruktur die, die Speicherung von mehreren Elementen erlaubt. Die wichtigen Eigenschaften einer Liste sind Ordnung, Veraenderbarkeit.</t>
   </si>
   <si>
     <t>Akronym UML</t>
   </si>
   <si>
-    <t>Wofuer steht UML? Gib die ausgeschriebene Version von der Abkuerzung  "UML"</t>
-  </si>
-  <si>
     <t>Wofuer steht die Abkuerzung UML?</t>
   </si>
   <si>
@@ -196,9 +151,6 @@
     <t>Programmieren UML</t>
   </si>
   <si>
-    <t>Welche Programmierart eignet sich besonders gut in Zusammenarbeit mit UML Diagrammen</t>
-  </si>
-  <si>
     <t>Angabe der Programmierart: Objektorientiert</t>
   </si>
   <si>
@@ -220,9 +172,6 @@
     <t>Definition higher order functions</t>
   </si>
   <si>
-    <t>Was ist eine Funktion hoeherer Ordnung? Gib eine kurze Definition</t>
-  </si>
-  <si>
     <t>Definition von Funktionen hoeherer Ordnung</t>
   </si>
   <si>
@@ -232,9 +181,6 @@
     <t>Definition Funktion</t>
   </si>
   <si>
-    <t>Was ist eine Funktion? Gib eine kurze Definition</t>
-  </si>
-  <si>
     <t>Definition von Funktionen</t>
   </si>
   <si>
@@ -244,12 +190,6 @@
     <t>Definition pure function</t>
   </si>
   <si>
-    <t>Was ist eine pure function</t>
-  </si>
-  <si>
-    <t>Definition von pure functions</t>
-  </si>
-  <si>
     <t>Eine pure function hat alle Eigenschaften einer normalen Funktion, allerdings muss diese im Wesentlichen zwei extra Bedingungen erfüllen: Determinismus und Abwesenheit von Nebenwirkungen.</t>
   </si>
   <si>
@@ -262,15 +202,9 @@
     <t>Definition von Interface</t>
   </si>
   <si>
-    <t>Ein Interface ist eine Art abstraker Klasse, welche einige abstrakte Methoden definiert, allerdings ohne diese zu implementieren.</t>
-  </si>
-  <si>
     <t>Keywords Vererbung</t>
   </si>
   <si>
-    <t>Welche beiden keywords verwendet Java fuer Vererbung</t>
-  </si>
-  <si>
     <t>Angabe der beiden Keywords: extends und implements</t>
   </si>
   <si>
@@ -280,21 +214,12 @@
     <t>Beispiele Operationen mit Zahlen</t>
   </si>
   <si>
-    <t>Welche Operationen mit Zahlen gibt es? Nenne mindestens 5 Beispiele</t>
-  </si>
-  <si>
-    <t>5 Beispiele fuer Operationen auf Zahlen</t>
-  </si>
-  <si>
     <t>Beispiele beinhalten + (Plus), - (Minus), * (Multiplikation), / (Division), % (Modulo)</t>
   </si>
   <si>
     <t>Definition primitive Datentypen</t>
   </si>
   <si>
-    <t>Was ist ein primitiver Datentyp? Gebe eine kurze Definition in eigenen Worten</t>
-  </si>
-  <si>
     <t>Definition: Was ist ein primitiver Datentyp</t>
   </si>
   <si>
@@ -304,9 +229,6 @@
     <t>Eigenschaften primitive Datentypen</t>
   </si>
   <si>
-    <t>Wie werden primitive Datentypen im Speicher abgelegt? Erkläre in eigenen Worten</t>
-  </si>
-  <si>
     <t>Erklärung: Wie werden primitive Datentypen im Speicher abgelegt?</t>
   </si>
   <si>
@@ -367,9 +289,6 @@
     <t>Welche Zugriffsarten für Klassen gibt es und was macht diese aus?</t>
   </si>
   <si>
-    <t>Welche Zugriffsarten gibt es fuer Klassenattribute in java</t>
-  </si>
-  <si>
     <t>Variablen und Funktionen können unterschiedliche Zugriffsarten haben, darunter private, public, protected</t>
   </si>
   <si>
@@ -379,9 +298,6 @@
     <t>Welche Arten von Attributen kann eine Klasse haben?</t>
   </si>
   <si>
-    <t>Arten: Welche Arten von Attributen kann eine Klasse haben</t>
-  </si>
-  <si>
     <t>Attribute koennen sowohl Variablen als auch Funktionen sein.</t>
   </si>
   <si>
@@ -412,9 +328,6 @@
     <t>Beispiele Datenstrukturen</t>
   </si>
   <si>
-    <t>Nenne mindestens 3 Beispiele für eine Datenstruktur</t>
-  </si>
-  <si>
     <t>Beispiele: Nenne mindestens 3 Beispiele fuer eine Datenstruktur</t>
   </si>
   <si>
@@ -424,9 +337,6 @@
     <t>Definition Exception</t>
   </si>
   <si>
-    <t>Was ist eine Exception? Gib eine kurze Definition in eigenen Worten</t>
-  </si>
-  <si>
     <t>Definition: Was ist eine Exception</t>
   </si>
   <si>
@@ -436,48 +346,24 @@
     <t>Arten Exceptions</t>
   </si>
   <si>
-    <t>Welche Arten von Exceptions gibt es in Java, nenne 3</t>
-  </si>
-  <si>
-    <t>Arten: Welche Arten von Exception gibt es in Java</t>
-  </si>
-  <si>
     <t>In Java gibt es sogenannte eingebaute checked- und unchecked- exceptions, als auch vom user definierte exceptions</t>
   </si>
   <si>
     <t>Was ist objektorientiertes Programmieren?</t>
   </si>
   <si>
-    <t>Was ist objektorientiertes Programmieren, gib eine kurze Definition in eigenen Worten.</t>
-  </si>
-  <si>
-    <t>Definition: Was ist objektorientiertes Programmierne</t>
-  </si>
-  <si>
     <t>Bei der objektorientierten Programmierung wird das gewuenschte Verhalten des Programms erreicht, indem man Objekte und ihr Verhalten definiert. Dies steht im Gegensatz zur Programmierung mit reiner Logik und Funktionen.</t>
   </si>
   <si>
     <t>Definition Map Funktion</t>
   </si>
   <si>
-    <t>Was ist die Map Funktion? Gib eine kurze Definition in eigenen Worten.</t>
-  </si>
-  <si>
-    <t>Definition: Was ist die map funktion (python)</t>
-  </si>
-  <si>
     <t>Die Map Funktion in python bekommt iterierbare Daten und eine Funktion als input. Die Funktion wird dann auf jedes Element der Daten angewendet. Rueckgabewert ist ein neues map Objekt mit den neuen Werten.</t>
   </si>
   <si>
     <t>Definition Filter</t>
   </si>
   <si>
-    <t>Was ist die Filter Funktion? Gib eine kurze Definition in eigenen Worten.</t>
-  </si>
-  <si>
-    <t>Definition: Was ist die filter funktion (python)</t>
-  </si>
-  <si>
     <t>Die Filter Funktion in python benoetigt eine iterierbare Datenstruktur und eine Bedingung. Diese Bedingung wird dann auf jedem Element in der Datenstruktur geprueft und basierend auf der Bedingung werden Elemente gefiltert und eine neue Datenstruktur wird erstellt.</t>
   </si>
   <si>
@@ -505,9 +391,6 @@
     <t>Definition Currying</t>
   </si>
   <si>
-    <t>Was ist Currying? Gib eine kurze Definition in eigenen Worten</t>
-  </si>
-  <si>
     <t>Definition: Was ist Currying</t>
   </si>
   <si>
@@ -526,9 +409,6 @@
     <t>Definition if/else</t>
   </si>
   <si>
-    <t>Was ist eine if/else Bedingung? Gib eine kurze Definition in eigenen Worten</t>
-  </si>
-  <si>
     <t>Definition: Was ist eine if/else Bedingung</t>
   </si>
   <si>
@@ -536,9 +416,6 @@
   </si>
   <si>
     <t>Code: Rekursion</t>
-  </si>
-  <si>
-    <t>Schaue dir die beiden Implementierungen zur Berechnung der Fibonacci Folge an? Welche der beiden ist iterativ und welche rekursiv, welche Implementierung ist besser geeignet und wieso?</t>
   </si>
   <si>
     <t>Welche der Implementierungen fib1 und fib2 ist rekursiv und welche ist iterativ? Welche der beiden ist die bessere Implementierung und warum?</t>
@@ -567,9 +444,6 @@
     <t>Code: Map</t>
   </si>
   <si>
-    <t>Was macht das folgende Codebeispiel? Lege besonders Wert auf die Funktion von Map</t>
-  </si>
-  <si>
     <t>Was  macht das folgende Code Snippet? Was ist result nach Ausfuehren?</t>
   </si>
   <si>
@@ -589,13 +463,190 @@
   </si>
   <si>
     <t>conceptNode</t>
+  </si>
+  <si>
+    <t>Beispiele Anweisungen</t>
+  </si>
+  <si>
+    <t>Gib drei Beispiele, wie Anweisungen in Python aussehen könnten.</t>
+  </si>
+  <si>
+    <t>Anweisungen wie "x = x*20" sind gefragt. Dies kann auch eine einfache Anweisung sein. Pro richtiger Anweisung gibt es einen Punkt.</t>
+  </si>
+  <si>
+    <t>x= 1, a = b und myVar = a*b</t>
+  </si>
+  <si>
+    <t>Operationen: Nenne zwei Operationen die man auf strings anwenden kann. Ein Punkt pro genanntem Operator.</t>
+  </si>
+  <si>
+    <t>Beispiele: Nenne jeweils zwei Beispiele fuer mutable/immutable Variablen. Einen halben Punkt pro richtigem Beispiel.</t>
+  </si>
+  <si>
+    <t>Definition: Wie funktioniert eine while loop</t>
+  </si>
+  <si>
+    <t>Ein while loop bekommt eine boolsche Bedingung die wiederholt geprueft werden kann. Solange diese Bedingung den Wert wahr hat wird ein Code Block ausgefuehrt bevor die Bedingung erneut geprueft wird.</t>
+  </si>
+  <si>
+    <t>Was ist eine Liste? Gib eine kurze Definition in eigenen Worten und nenne zwei Eigenschaften.</t>
+  </si>
+  <si>
+    <t>Definition: Was ist eine Liste. Ein Punkt für die richtige Definition, zwei Punkte für die Nennung der Eigenschaften.</t>
+  </si>
+  <si>
+    <t>Welche Programmierart eignet sich besonders gut in Zusammenarbeit mit UML Diagrammen?</t>
+  </si>
+  <si>
+    <t>Wie funktioniert eine while loop? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Was sind Strings? Beschreibe Strings in eigenen Worten und gebe eine kurze Definition (1-2 Saetze).</t>
+  </si>
+  <si>
+    <t>Welchen Vorteil von Rekursion haben wir kennengelernt? Nenne einen Vorteil aus der Vorlesung.</t>
+  </si>
+  <si>
+    <t>Was ist ein Tupel? Gib eine kurze Definition.</t>
+  </si>
+  <si>
+    <t>Wie definiert man ein Tupel? Schreibe ein Tupel mit den Elementen 3, 7 und 5 auf (in dieser Reihenfolge).</t>
+  </si>
+  <si>
+    <t>Was ist eine Funktion? Gib eine kurze Definition.</t>
+  </si>
+  <si>
+    <t>Was ist eine pure function?</t>
+  </si>
+  <si>
+    <t>Definition von pure functions. Ein Punkt für die Definition, ein Punkt für die zu erfüllenden Bedingungen.</t>
+  </si>
+  <si>
+    <t>Ein Interface ist eine Art abstrakte Klasse, welche einige abstrakte Methoden definiert, allerdings ohne diese zu implementieren.</t>
+  </si>
+  <si>
+    <t>Welche beiden keywords verwendet Java für Vererbung?</t>
+  </si>
+  <si>
+    <t>Gib ein Beispiel für einen String. Wie macht man einen String im Programmcode kenntlich?</t>
+  </si>
+  <si>
+    <t>Welche Methoden gibt es für strings in python? Nenne mindestens zwei.</t>
+  </si>
+  <si>
+    <t>Nenne jeweils zwei Beispiele für mutable/immutable Variablen in Python.</t>
+  </si>
+  <si>
+    <t>Wofuer steht UML? Gib die ausgeschriebene Version von der Abkürzung "UML".</t>
+  </si>
+  <si>
+    <t>Was ist eine Funktion höherer Ordnung? Gib eine kurze Definition.</t>
+  </si>
+  <si>
+    <t>Welche Operationen mit Zahlen gibt es? Nenne mindestens 5 Beispiele.</t>
+  </si>
+  <si>
+    <t>5 Beispiele fuer Operationen auf Zahlen. Ein Punkt pro richtigem Beispiel.</t>
+  </si>
+  <si>
+    <t>Was ist ein primitiver Datentyp? Gebe eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Wie werden primitive Datentypen im Speicher abgelegt? Erkläre in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Welche Zugriffsarten gibt es fuer Klassenattribute in java? Ein Punkt pro richtig genannter Zugriffsart.</t>
+  </si>
+  <si>
+    <t>Arten: Welche Arten von Attributen kann eine Klasse haben. Ein Punkt pro Art.</t>
+  </si>
+  <si>
+    <t>Was ist eine Exception? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Nenne mindestens 3 Beispiele für eine Datenstruktur.</t>
+  </si>
+  <si>
+    <t>Welche Arten von Exceptions gibt es in Java? Nenne 3.</t>
+  </si>
+  <si>
+    <t>Arten: Welche Arten von Exception gibt es in Java? Ein Punkt pro Art.</t>
+  </si>
+  <si>
+    <t>Definition: Was ist objektorientiertes Programmieren</t>
+  </si>
+  <si>
+    <t>Was ist objektorientiertes Programmieren? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Was ist die Map Funktion? Was gibt sie zurück? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Definition: Was ist die map funktion (python). Ein Punkt für die Definition, ein Punkt für die Rückgabe.</t>
+  </si>
+  <si>
+    <t>Was ist die Filter Funktion? Was macht sie? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Definition: Was ist die filter funktion (python). Ein Punkt für die Definition, ein Punkt für die Funktionsweise.</t>
+  </si>
+  <si>
+    <t>Was ist Currying? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Wie funktioniert eine for loop? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Was ist eine if/else Bedingung? Gib eine kurze Definition in eigenen Worten.</t>
+  </si>
+  <si>
+    <t>Schaue dir die beiden Implementierungen zur Berechnung der Fibonacci Folge an. Welche der beiden ist iterativ und welche rekursiv, welche Implementierung ist besser geeignet und wieso?</t>
+  </si>
+  <si>
+    <t>Was macht das folgende Codebeispiel? Lege besonders Wert auf die Funktion von Map.</t>
+  </si>
+  <si>
+    <t>Warum gibt (3.0*0.1 == 0.3) false aus und was bedeutet das für die Programmierung?</t>
+  </si>
+  <si>
+    <t>Dieses Statement gibt false aus, da beim rechnen mit Gleitkommazahlen gewisse Rundungsfehler auftreten können. Dies sollte man beim Programmieren beachten und in diesem Fall beispielsweise mit einem Differenzvergleich arbeiten oder entsprechende Pakete installieren.</t>
+  </si>
+  <si>
+    <t>1 Punkt für die Beschreibung der Ursache, 1 Punkt dafür, wie man damit umgehen kann.</t>
+  </si>
+  <si>
+    <t>Typenumwandlung</t>
+  </si>
+  <si>
+    <t>Es gibt die Variable a="Meine Zahlen: ", b=3 und c=5.8. Würde print(a+b+c) funktionieren? Wenn nicht, warum nicht? Was müsste verändert werden?</t>
+  </si>
+  <si>
+    <t>1 Punkt für die richtige Erkenntnis, dass der Befehl nicht funkioniert. 1 Punkt für die Erklärung, warum. 1 Punkt für die richtige Verbesserung.</t>
+  </si>
+  <si>
+    <t>Nein, der Befehl würde so nicht funktionieren, weil zwei der Variablen kein String sind. Ein funktionierender Befehl wäre: print(a+str(b)+str(c)).</t>
+  </si>
+  <si>
+    <t>Gleitkommazahlen</t>
+  </si>
+  <si>
+    <t>Vor- und Nachteile</t>
+  </si>
+  <si>
+    <t>Welche Vor- und Nachteile bezüglich der dynamischen Typisierung fallen dir ein? Nenne jeweils zwei.</t>
+  </si>
+  <si>
+    <t>Vorteile: Man bleibt flexibel und kann schneller Entwickeln. Außerdem kann Code leichter umstrukturiert werden. Nachteile: Fehler treten teilweise erst sehr spät, also beispielsweise in der Laufzeit, auf. Diese lassen sich schwerer beheben. Außerdem werden IDEs eingeschränkt, da sie weniger Informationen über den Code erlangen und dadurch Probleme bei der automatischen Codevervollständigung haben können.</t>
+  </si>
+  <si>
+    <t>1 Punkt pro Vor- oder Nachteil. Es müssen nicht dieselben Aspekte genannt werden, wie in der Musterlöung. Solange plausibel und sinngemäß, sollen auch Punkte vergeben werden. Es müssen zwei Vorteile und zwei Nachteile sein.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -629,12 +680,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -675,7 +720,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -686,16 +731,28 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -914,24 +971,25 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I49"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.5" customWidth="1"/>
-    <col min="3" max="4" width="19" customWidth="1"/>
-    <col min="5" max="5" width="17.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="47" customWidth="1"/>
-    <col min="8" max="8" width="89.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20.875" customWidth="1"/>
+    <col min="2" max="2" width="25.625" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="94.5" customWidth="1"/>
+    <col min="5" max="5" width="17.875" customWidth="1"/>
+    <col min="6" max="6" width="18.875" customWidth="1"/>
+    <col min="7" max="7" width="66.5" style="10" customWidth="1"/>
+    <col min="8" max="8" width="100.375" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>182</v>
+        <v>140</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -943,16 +1001,16 @@
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="G1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="G1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>9</v>
       </c>
@@ -960,103 +1018,103 @@
         <v>5</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="3">
+        <v>2</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="3">
-        <v>2</v>
-      </c>
-      <c r="F2" s="3">
-        <v>1</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="E3" s="3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3">
+        <v>2</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="4" t="s">
+      <c r="H3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="3">
-        <v>2</v>
-      </c>
-      <c r="F3" s="3">
-        <v>1</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3">
         <v>1</v>
       </c>
       <c r="F4" s="3">
-        <v>1</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>164</v>
       </c>
       <c r="E5" s="3">
         <v>1</v>
       </c>
       <c r="F5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E6" s="3">
         <v>2</v>
@@ -1065,22 +1123,22 @@
         <v>1</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>34</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="4" t="s">
-        <v>26</v>
+      <c r="D7" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="E7" s="3">
         <v>1</v>
@@ -1089,22 +1147,22 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>41</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="4" t="s">
-        <v>30</v>
+      <c r="D8" s="8" t="s">
+        <v>156</v>
       </c>
       <c r="E8" s="3">
         <v>2</v>
@@ -1113,22 +1171,22 @@
         <v>1</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>41</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="4" t="s">
-        <v>34</v>
+      <c r="D9" s="8" t="s">
+        <v>157</v>
       </c>
       <c r="E9" s="3">
         <v>1</v>
@@ -1137,22 +1195,22 @@
         <v>1</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>30</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E10" s="3">
         <v>2</v>
@@ -1161,94 +1219,94 @@
         <v>1</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>30</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="4" t="s">
-        <v>42</v>
+      <c r="D11" s="8" t="s">
+        <v>165</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
       </c>
       <c r="F11" s="3">
-        <v>1</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>21</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E12" s="9">
-        <v>2</v>
-      </c>
-      <c r="F12" s="9">
-        <v>1</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E12" s="7">
+        <v>2</v>
+      </c>
+      <c r="F12" s="7">
+        <v>1</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>40</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E13" s="9">
-        <v>1</v>
-      </c>
-      <c r="F13" s="9">
-        <v>1</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E13" s="7">
+        <v>1</v>
+      </c>
+      <c r="F13" s="7">
+        <v>3</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>85</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="4" t="s">
-        <v>54</v>
+      <c r="D14" s="8" t="s">
+        <v>166</v>
       </c>
       <c r="E14" s="3">
         <v>1</v>
@@ -1257,22 +1315,22 @@
         <v>1</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>85</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="4" t="s">
-        <v>58</v>
+      <c r="D15" s="8" t="s">
+        <v>152</v>
       </c>
       <c r="E15" s="3">
         <v>1</v>
@@ -1281,22 +1339,22 @@
         <v>1</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>64</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="4" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E16" s="3">
         <v>2</v>
@@ -1305,22 +1363,22 @@
         <v>1</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>28</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="C17" s="3"/>
-      <c r="D17" s="4" t="s">
-        <v>66</v>
+      <c r="D17" s="8" t="s">
+        <v>167</v>
       </c>
       <c r="E17" s="3">
         <v>2</v>
@@ -1329,22 +1387,22 @@
         <v>1</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>23</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="C18" s="3"/>
-      <c r="D18" s="4" t="s">
-        <v>70</v>
+      <c r="D18" s="8" t="s">
+        <v>158</v>
       </c>
       <c r="E18" s="3">
         <v>2</v>
@@ -1353,46 +1411,46 @@
         <v>1</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>32</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
       <c r="C19" s="3"/>
-      <c r="D19" s="4" t="s">
-        <v>74</v>
+      <c r="D19" s="8" t="s">
+        <v>159</v>
       </c>
       <c r="E19" s="3">
         <v>2</v>
       </c>
       <c r="F19" s="3">
-        <v>1</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>96</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="4" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="E20" s="3">
         <v>2</v>
@@ -1401,70 +1459,70 @@
         <v>1</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>93</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="C21" s="3"/>
-      <c r="D21" s="4" t="s">
-        <v>82</v>
+      <c r="D21" s="8" t="s">
+        <v>162</v>
       </c>
       <c r="E21" s="3">
         <v>1</v>
       </c>
       <c r="F21" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>14</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="C22" s="3"/>
-      <c r="D22" s="4" t="s">
-        <v>86</v>
+      <c r="D22" s="8" t="s">
+        <v>168</v>
       </c>
       <c r="E22" s="3">
         <v>1</v>
       </c>
       <c r="F22" s="3">
-        <v>1</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>8</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7" t="s">
-        <v>90</v>
+      <c r="B23" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5" t="s">
+        <v>170</v>
       </c>
       <c r="E23" s="3">
         <v>2</v>
@@ -1472,23 +1530,23 @@
       <c r="F23" s="3">
         <v>1</v>
       </c>
-      <c r="G23" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G23" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>8</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7" t="s">
-        <v>94</v>
+      <c r="B24" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5" t="s">
+        <v>171</v>
       </c>
       <c r="E24" s="3">
         <v>2</v>
@@ -1496,23 +1554,23 @@
       <c r="F24" s="3">
         <v>1</v>
       </c>
-      <c r="G24" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G24" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H24" s="10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>83</v>
       </c>
-      <c r="B25" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7" t="s">
-        <v>98</v>
+      <c r="B25" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5" t="s">
+        <v>72</v>
       </c>
       <c r="E25" s="3">
         <v>2</v>
@@ -1520,23 +1578,23 @@
       <c r="F25" s="3">
         <v>1</v>
       </c>
-      <c r="G25" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G25" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>83</v>
       </c>
-      <c r="B26" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7" t="s">
-        <v>102</v>
+      <c r="B26" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="E26" s="3">
         <v>1</v>
@@ -1544,47 +1602,47 @@
       <c r="F26" s="3">
         <v>1</v>
       </c>
-      <c r="G26" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G26" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>12</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7" t="s">
-        <v>106</v>
+      <c r="B27" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="E27" s="3">
         <v>5</v>
       </c>
       <c r="F27" s="3">
-        <v>1</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>86</v>
       </c>
-      <c r="B28" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7" t="s">
-        <v>110</v>
+      <c r="B28" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5" t="s">
+        <v>84</v>
       </c>
       <c r="E28" s="3">
         <v>2</v>
@@ -1592,71 +1650,71 @@
       <c r="F28" s="3">
         <v>1</v>
       </c>
-      <c r="G28" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G28" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>86</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7" t="s">
-        <v>114</v>
+      <c r="B29" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5" t="s">
+        <v>88</v>
       </c>
       <c r="E29" s="3">
         <v>2</v>
       </c>
       <c r="F29" s="3">
-        <v>1</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="H29" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>86</v>
       </c>
-      <c r="B30" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7" t="s">
-        <v>118</v>
+      <c r="B30" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="E30" s="3">
         <v>1</v>
       </c>
       <c r="F30" s="3">
-        <v>1</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>99</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7" t="s">
-        <v>122</v>
+      <c r="B31" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5" t="s">
+        <v>94</v>
       </c>
       <c r="E31" s="3">
         <v>2</v>
@@ -1664,71 +1722,71 @@
       <c r="F31" s="3">
         <v>1</v>
       </c>
-      <c r="G31" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G31" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H31" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>39</v>
       </c>
-      <c r="B32" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7" t="s">
-        <v>126</v>
+      <c r="B32" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5" t="s">
+        <v>98</v>
       </c>
       <c r="E32" s="3">
         <v>2</v>
       </c>
       <c r="F32" s="3">
-        <v>1</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>39</v>
       </c>
-      <c r="B33" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7" t="s">
-        <v>130</v>
+      <c r="B33" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5" t="s">
+        <v>175</v>
       </c>
       <c r="E33" s="3">
         <v>1</v>
       </c>
       <c r="F33" s="3">
-        <v>1</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>101</v>
       </c>
-      <c r="B34" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7" t="s">
-        <v>134</v>
+      <c r="B34" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5" t="s">
+        <v>174</v>
       </c>
       <c r="E34" s="3">
         <v>2</v>
@@ -1736,47 +1794,47 @@
       <c r="F34" s="3">
         <v>1</v>
       </c>
-      <c r="G34" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="H34" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G34" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>101</v>
       </c>
-      <c r="B35" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7" t="s">
-        <v>138</v>
+      <c r="B35" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5" t="s">
+        <v>176</v>
       </c>
       <c r="E35" s="3">
         <v>1</v>
       </c>
       <c r="F35" s="3">
-        <v>1</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>73</v>
       </c>
-      <c r="B36" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7" t="s">
-        <v>142</v>
+      <c r="B36" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5" t="s">
+        <v>179</v>
       </c>
       <c r="E36" s="3">
         <v>2</v>
@@ -1784,71 +1842,71 @@
       <c r="F36" s="3">
         <v>1</v>
       </c>
-      <c r="G36" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G36" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
-      <c r="B37" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7" t="s">
-        <v>146</v>
+      <c r="B37" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5" t="s">
+        <v>180</v>
       </c>
       <c r="E37" s="3">
         <v>2</v>
       </c>
       <c r="F37" s="3">
-        <v>1</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
-      <c r="B38" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7" t="s">
-        <v>150</v>
+      <c r="B38" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5" t="s">
+        <v>182</v>
       </c>
       <c r="E38" s="3">
         <v>2</v>
       </c>
       <c r="F38" s="3">
-        <v>1</v>
-      </c>
-      <c r="G38" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
-      <c r="B39" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7" t="s">
-        <v>154</v>
+      <c r="B39" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5" t="s">
+        <v>116</v>
       </c>
       <c r="E39" s="3">
         <v>2</v>
@@ -1856,21 +1914,21 @@
       <c r="F39" s="3">
         <v>1</v>
       </c>
-      <c r="G39" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="H39" s="5"/>
-    </row>
-    <row r="40" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G39" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="H39" s="10"/>
+    </row>
+    <row r="40" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>8</v>
       </c>
-      <c r="B40" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7" t="s">
-        <v>157</v>
+      <c r="B40" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="E40" s="3">
         <v>2</v>
@@ -1878,140 +1936,233 @@
       <c r="F40" s="3">
         <v>1</v>
       </c>
-      <c r="G40" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G40" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>33</v>
       </c>
-      <c r="B41" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="E41" s="9">
-        <v>1</v>
-      </c>
-      <c r="F41" s="9">
-        <v>1</v>
-      </c>
-      <c r="G41" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="E41" s="7">
+        <v>1</v>
+      </c>
+      <c r="F41" s="7">
+        <v>1</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>22</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E42" s="9">
-        <v>1</v>
-      </c>
-      <c r="F42" s="9">
-        <v>1</v>
-      </c>
-      <c r="G42" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="E42" s="7">
+        <v>1</v>
+      </c>
+      <c r="F42" s="7">
+        <v>1</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>19</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="E43" s="9">
-        <v>1</v>
-      </c>
-      <c r="F43" s="9">
-        <v>1</v>
-      </c>
-      <c r="G43" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H43" s="5" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="E43" s="7">
+        <v>1</v>
+      </c>
+      <c r="F43" s="7">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>34</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7" t="s">
-        <v>172</v>
+      <c r="B44" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5" t="s">
+        <v>187</v>
       </c>
       <c r="E44" s="3">
         <v>5</v>
       </c>
       <c r="F44" s="3">
-        <v>1</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>173</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>174</v>
+        <v>3</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>133</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>36</v>
       </c>
-      <c r="B45" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7" t="s">
-        <v>177</v>
+      <c r="B45" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5" t="s">
+        <v>188</v>
       </c>
       <c r="E45" s="3">
         <v>4</v>
       </c>
       <c r="F45" s="3">
-        <v>1</v>
-      </c>
-      <c r="G45" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="H45" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="I45" s="8" t="s">
-        <v>180</v>
+        <v>2</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A46" s="7">
+        <v>7</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E46" s="7">
+        <v>2</v>
+      </c>
+      <c r="F46" s="7">
+        <v>3</v>
+      </c>
+      <c r="G46" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>13</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="E47" s="7">
+        <v>2</v>
+      </c>
+      <c r="F47">
+        <v>2</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="H47" s="12" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>15</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="E48">
+        <v>2</v>
+      </c>
+      <c r="F48">
+        <v>3</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="H48" s="12" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="63" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>6</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="E49">
+        <v>4</v>
+      </c>
+      <c r="F49">
+        <v>4</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="H49" s="12" t="s">
+        <v>199</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added 4 new freetext tasks to kompetenzraster
Bug: Cant see the last one in the graph
</commit_message>
<xml_diff>
--- a/files/freetext_questions.xlsx
+++ b/files/freetext_questions.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jan\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226ACC4B-B604-46CC-90BD-965543519A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE4DDE6-A867-4C6A-8A0B-D5E8292CD4A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -738,16 +738,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2094,7 +2094,7 @@
     </row>
     <row r="47" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>196</v>

</xml_diff>

<commit_message>
updated Kompetenzraster / changed some score and conceptNode of questions
</commit_message>
<xml_diff>
--- a/files/freetext_questions.xlsx
+++ b/files/freetext_questions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcsauer/GitHub/hefl/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE4DDE6-A867-4C6A-8A0B-D5E8292CD4A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D837040B-3A1A-0D4F-AC00-E50716F2FC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -504,15 +504,9 @@
     <t>Was sind Strings? Beschreibe Strings in eigenen Worten und gebe eine kurze Definition (1-2 Saetze).</t>
   </si>
   <si>
-    <t>Welchen Vorteil von Rekursion haben wir kennengelernt? Nenne einen Vorteil aus der Vorlesung.</t>
-  </si>
-  <si>
     <t>Was ist ein Tupel? Gib eine kurze Definition.</t>
   </si>
   <si>
-    <t>Wie definiert man ein Tupel? Schreibe ein Tupel mit den Elementen 3, 7 und 5 auf (in dieser Reihenfolge).</t>
-  </si>
-  <si>
     <t>Was ist eine Funktion? Gib eine kurze Definition.</t>
   </si>
   <si>
@@ -640,17 +634,30 @@
   </si>
   <si>
     <t>1 Punkt pro Vor- oder Nachteil. Es müssen nicht dieselben Aspekte genannt werden, wie in der Musterlöung. Solange plausibel und sinngemäß, sollen auch Punkte vergeben werden. Es müssen zwei Vorteile und zwei Nachteile sein.</t>
+  </si>
+  <si>
+    <t>Wie deklariert man ein Tupel? Schreibe ein Tupel mit den Elementen 3, 7 und 5 auf (in dieser Reihenfolge).</t>
+  </si>
+  <si>
+    <t>Welchen Vorteil von Rekursion haben wir kennengelernt? Nenne ein Beispiel aus der Vorlesung.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -720,25 +727,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -747,10 +754,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -972,19 +982,19 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:I49"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.875" customWidth="1"/>
-    <col min="2" max="2" width="25.625" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
     <col min="4" max="4" width="94.5" customWidth="1"/>
-    <col min="5" max="5" width="17.875" customWidth="1"/>
-    <col min="6" max="6" width="18.875" customWidth="1"/>
+    <col min="5" max="5" width="17.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="66.5" style="10" customWidth="1"/>
-    <col min="8" max="8" width="100.375" style="11" customWidth="1"/>
+    <col min="8" max="8" width="100.33203125" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>141</v>
       </c>
@@ -1010,7 +1020,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>9</v>
       </c>
@@ -1025,7 +1035,7 @@
         <v>2</v>
       </c>
       <c r="F2" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>6</v>
@@ -1034,7 +1044,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>9</v>
       </c>
@@ -1043,7 +1053,7 @@
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E3" s="3">
         <v>2</v>
@@ -1058,7 +1068,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>9</v>
       </c>
@@ -1082,7 +1092,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>9</v>
       </c>
@@ -1090,7 +1100,7 @@
         <v>14</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E5" s="3">
         <v>1</v>
@@ -1105,7 +1115,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>34</v>
       </c>
@@ -1117,7 +1127,7 @@
         <v>18</v>
       </c>
       <c r="E6" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="3">
         <v>1</v>
@@ -1129,7 +1139,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>34</v>
       </c>
@@ -1137,11 +1147,11 @@
         <v>21</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="8" t="s">
-        <v>155</v>
+      <c r="D7" s="14" t="s">
+        <v>200</v>
       </c>
       <c r="E7" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="3">
         <v>1</v>
@@ -1153,7 +1163,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>41</v>
       </c>
@@ -1162,10 +1172,10 @@
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E8" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
@@ -1177,7 +1187,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>41</v>
       </c>
@@ -1185,23 +1195,23 @@
         <v>27</v>
       </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="8" t="s">
-        <v>157</v>
+      <c r="D9" s="14" t="s">
+        <v>199</v>
       </c>
       <c r="E9" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="14" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>30</v>
       </c>
@@ -1225,7 +1235,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>30</v>
       </c>
@@ -1234,7 +1244,7 @@
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
@@ -1249,7 +1259,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>21</v>
       </c>
@@ -1273,7 +1283,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>40</v>
       </c>
@@ -1285,7 +1295,7 @@
         <v>150</v>
       </c>
       <c r="E13" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="7">
         <v>3</v>
@@ -1297,7 +1307,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>85</v>
       </c>
@@ -1306,7 +1316,7 @@
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E14" s="3">
         <v>1</v>
@@ -1321,7 +1331,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>85</v>
       </c>
@@ -1345,7 +1355,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>64</v>
       </c>
@@ -1369,7 +1379,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>28</v>
       </c>
@@ -1378,7 +1388,7 @@
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E17" s="3">
         <v>2</v>
@@ -1393,7 +1403,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>23</v>
       </c>
@@ -1402,7 +1412,7 @@
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E18" s="3">
         <v>2</v>
@@ -1417,7 +1427,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>32</v>
       </c>
@@ -1426,7 +1436,7 @@
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E19" s="3">
         <v>2</v>
@@ -1435,13 +1445,13 @@
         <v>2</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>96</v>
       </c>
@@ -1462,10 +1472,10 @@
         <v>59</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>93</v>
       </c>
@@ -1474,7 +1484,7 @@
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E21" s="3">
         <v>1</v>
@@ -1489,7 +1499,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>14</v>
       </c>
@@ -1498,7 +1508,7 @@
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E22" s="3">
         <v>1</v>
@@ -1507,13 +1517,13 @@
         <v>5</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>8</v>
       </c>
@@ -1522,10 +1532,10 @@
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E23" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="3">
         <v>1</v>
@@ -1537,7 +1547,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>8</v>
       </c>
@@ -1546,10 +1556,10 @@
       </c>
       <c r="C24" s="5"/>
       <c r="D24" s="5" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E24" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="3">
         <v>1</v>
@@ -1561,7 +1571,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>83</v>
       </c>
@@ -1585,7 +1595,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>83</v>
       </c>
@@ -1609,7 +1619,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>12</v>
       </c>
@@ -1633,7 +1643,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>86</v>
       </c>
@@ -1657,7 +1667,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>86</v>
       </c>
@@ -1675,13 +1685,13 @@
         <v>3</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H29" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>86</v>
       </c>
@@ -1699,13 +1709,13 @@
         <v>2</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H30" s="10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>99</v>
       </c>
@@ -1729,7 +1739,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>39</v>
       </c>
@@ -1753,7 +1763,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>39</v>
       </c>
@@ -1762,7 +1772,7 @@
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E33" s="3">
         <v>1</v>
@@ -1777,7 +1787,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>101</v>
       </c>
@@ -1786,7 +1796,7 @@
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E34" s="3">
         <v>2</v>
@@ -1801,7 +1811,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>101</v>
       </c>
@@ -1810,7 +1820,7 @@
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E35" s="3">
         <v>1</v>
@@ -1819,13 +1829,13 @@
         <v>3</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H35" s="10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>73</v>
       </c>
@@ -1834,7 +1844,7 @@
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E36" s="3">
         <v>2</v>
@@ -1843,13 +1853,13 @@
         <v>1</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H36" s="10" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -1858,7 +1868,7 @@
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E37" s="3">
         <v>2</v>
@@ -1867,13 +1877,13 @@
         <v>2</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H37" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -1882,7 +1892,7 @@
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E38" s="3">
         <v>2</v>
@@ -1891,13 +1901,13 @@
         <v>2</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H38" s="10" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -1909,7 +1919,7 @@
         <v>116</v>
       </c>
       <c r="E39" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" s="3">
         <v>1</v>
@@ -1919,7 +1929,7 @@
       </c>
       <c r="H39" s="10"/>
     </row>
-    <row r="40" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>8</v>
       </c>
@@ -1931,7 +1941,7 @@
         <v>119</v>
       </c>
       <c r="E40" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" s="3">
         <v>1</v>
@@ -1943,7 +1953,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>33</v>
       </c>
@@ -1952,7 +1962,7 @@
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E41" s="7">
         <v>1</v>
@@ -1967,7 +1977,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>22</v>
       </c>
@@ -1976,7 +1986,7 @@
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E42" s="7">
         <v>1</v>
@@ -1991,7 +2001,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>19</v>
       </c>
@@ -2000,7 +2010,7 @@
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E43" s="7">
         <v>1</v>
@@ -2015,7 +2025,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>34</v>
       </c>
@@ -2024,7 +2034,7 @@
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E44" s="3">
         <v>5</v>
@@ -2042,7 +2052,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>36</v>
       </c>
@@ -2051,7 +2061,7 @@
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E45" s="3">
         <v>4</v>
@@ -2069,7 +2079,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" s="7">
         <v>7</v>
       </c>
@@ -2092,38 +2102,38 @@
         <v>145</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>12</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D47" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E47" s="7">
+        <v>2</v>
+      </c>
+      <c r="F47">
+        <v>2</v>
+      </c>
+      <c r="G47" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="E47" s="7">
-        <v>2</v>
-      </c>
-      <c r="F47">
-        <v>2</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>191</v>
-      </c>
       <c r="H47" s="12" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>15</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E48">
         <v>2</v>
@@ -2132,21 +2142,21 @@
         <v>3</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H48" s="12" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" ht="63" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>6</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E49">
         <v>4</v>
@@ -2155,10 +2165,10 @@
         <v>4</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H49" s="12" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updatet java part of the graph
</commit_message>
<xml_diff>
--- a/files/freetext_questions.xlsx
+++ b/files/freetext_questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcsauer/GitHub/hefl/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D837040B-3A1A-0D4F-AC00-E50716F2FC01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA714BE7-EAAA-7343-9AF4-591247BD821D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1020,111 +1020,110 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
-        <v>9</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="E2" s="3">
-        <v>2</v>
-      </c>
-      <c r="F2" s="3">
-        <v>2</v>
-      </c>
-      <c r="G2" s="4" t="s">
+    <row r="2" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>6</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="B2" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A3" s="7">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>9</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="E3" s="7">
+        <v>2</v>
+      </c>
+      <c r="F3" s="7">
+        <v>3</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
         <v>8</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="E3" s="3">
-        <v>2</v>
-      </c>
-      <c r="F3" s="3">
-        <v>2</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A4" s="2">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="4" t="s">
-        <v>12</v>
+      <c r="B4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5" t="s">
+        <v>168</v>
       </c>
       <c r="E4" s="3">
         <v>1</v>
       </c>
       <c r="F4" s="3">
-        <v>2</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>146</v>
+        <v>1</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
-        <v>9</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>162</v>
+      <c r="A5" s="3">
+        <v>8</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5" t="s">
+        <v>169</v>
       </c>
       <c r="E5" s="3">
         <v>1</v>
       </c>
       <c r="F5" s="3">
-        <v>2</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="2">
-        <v>34</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="4" t="s">
-        <v>18</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>8</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="E6" s="3">
         <v>1</v>
@@ -1132,278 +1131,275 @@
       <c r="F6" s="3">
         <v>1</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>19</v>
+      <c r="G6" s="5" t="s">
+        <v>120</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>20</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="14" t="s">
-        <v>200</v>
+      <c r="D7" s="8" t="s">
+        <v>154</v>
       </c>
       <c r="E7" s="3">
         <v>2</v>
       </c>
       <c r="F7" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="8" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="E8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="14" t="s">
-        <v>199</v>
+      <c r="D9" s="4" t="s">
+        <v>12</v>
       </c>
       <c r="E9" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" s="3">
         <v>2</v>
       </c>
-      <c r="G9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="G9" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="4" t="s">
-        <v>31</v>
+        <v>14</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>162</v>
       </c>
       <c r="E10" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
-        <v>30</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="8" t="s">
-        <v>163</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>12</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="E11" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F11" s="3">
         <v>2</v>
       </c>
-      <c r="G11" s="8" t="s">
-        <v>147</v>
+      <c r="G11" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E12" s="7">
+        <v>2</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>14</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3">
+        <v>5</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>15</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>3</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>19</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="E15" s="7">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7">
+        <v>1</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
         <v>21</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B16" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5" t="s">
+      <c r="C16" s="5"/>
+      <c r="D16" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="E12" s="7">
-        <v>2</v>
-      </c>
-      <c r="F12" s="7">
-        <v>1</v>
-      </c>
-      <c r="G12" s="5" t="s">
+      <c r="E16" s="7">
+        <v>2</v>
+      </c>
+      <c r="F16" s="7">
+        <v>1</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H16" s="8" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
-        <v>40</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="E13" s="7">
-        <v>2</v>
-      </c>
-      <c r="F13" s="7">
-        <v>3</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="2">
-        <v>85</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="E14" s="3">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3">
-        <v>1</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
-        <v>85</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="E15" s="3">
-        <v>1</v>
-      </c>
-      <c r="F15" s="3">
-        <v>1</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
-        <v>64</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="3">
-        <v>2</v>
-      </c>
-      <c r="F16" s="3">
-        <v>1</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H16" s="10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
-        <v>28</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="3"/>
-      <c r="D17" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="E17" s="3">
-        <v>2</v>
-      </c>
-      <c r="F17" s="3">
-        <v>1</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>50</v>
+    <row r="17" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>22</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E17" s="7">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7">
+        <v>1</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>126</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>23</v>
       </c>
@@ -1427,40 +1423,40 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="E19" s="3">
         <v>2</v>
       </c>
       <c r="F19" s="3">
-        <v>2</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>158</v>
+        <v>1</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>50</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="4" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="E20" s="3">
         <v>2</v>
@@ -1469,22 +1465,22 @@
         <v>1</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>93</v>
+        <v>30</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="8" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E21" s="3">
         <v>1</v>
@@ -1492,71 +1488,71 @@
       <c r="F21" s="3">
         <v>2</v>
       </c>
-      <c r="G21" s="4" t="s">
-        <v>61</v>
+      <c r="G21" s="8" t="s">
+        <v>147</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="8" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="E22" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>65</v>
+        <v>122</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="E23" s="3">
-        <v>1</v>
-      </c>
-      <c r="F23" s="3">
+        <v>182</v>
+      </c>
+      <c r="E23" s="7">
+        <v>1</v>
+      </c>
+      <c r="F23" s="7">
         <v>1</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>66</v>
+        <v>123</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
-        <v>8</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5" t="s">
-        <v>169</v>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>34</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="3"/>
+      <c r="D24" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="E24" s="3">
         <v>1</v>
@@ -1564,23 +1560,23 @@
       <c r="F24" s="3">
         <v>1</v>
       </c>
-      <c r="G24" s="5" t="s">
-        <v>69</v>
+      <c r="G24" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="H24" s="10" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
-        <v>83</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5" t="s">
-        <v>72</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
+        <v>34</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" s="3"/>
+      <c r="D25" s="14" t="s">
+        <v>200</v>
       </c>
       <c r="E25" s="3">
         <v>2</v>
@@ -1588,335 +1584,339 @@
       <c r="F25" s="3">
         <v>1</v>
       </c>
-      <c r="G25" s="5" t="s">
-        <v>73</v>
+      <c r="G25" s="4" t="s">
+        <v>22</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>75</v>
+        <v>131</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5" t="s">
-        <v>76</v>
+        <v>185</v>
       </c>
       <c r="E26" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F26" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>77</v>
+        <v>132</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="C27" s="5"/>
       <c r="D27" s="5" t="s">
-        <v>80</v>
+        <v>178</v>
       </c>
       <c r="E27" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F27" s="3">
         <v>2</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>81</v>
+        <v>179</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
-        <v>86</v>
+        <v>36</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>83</v>
+        <v>135</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>84</v>
+        <v>186</v>
       </c>
       <c r="E28" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F28" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>85</v>
+        <v>136</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+        <v>137</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
-        <v>86</v>
+        <v>37</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="C29" s="5"/>
       <c r="D29" s="5" t="s">
-        <v>88</v>
+        <v>180</v>
       </c>
       <c r="E29" s="3">
         <v>2</v>
       </c>
       <c r="F29" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="5" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="E30" s="3">
         <v>1</v>
       </c>
       <c r="F30" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="H30" s="10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+      <c r="H30" s="10"/>
+    </row>
+    <row r="31" spans="1:9" ht="51" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
-        <v>99</v>
+        <v>39</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="E31" s="3">
         <v>2</v>
       </c>
       <c r="F31" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>39</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5" t="s">
-        <v>98</v>
+        <v>173</v>
       </c>
       <c r="E32" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>101</v>
+        <v>37</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="E33" s="3">
-        <v>1</v>
-      </c>
-      <c r="F33" s="3">
+        <v>150</v>
+      </c>
+      <c r="E33" s="7">
+        <v>2</v>
+      </c>
+      <c r="F33" s="7">
         <v>3</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>102</v>
+        <v>151</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A34" s="3">
-        <v>101</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5" t="s">
-        <v>172</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A34" s="2">
+        <v>41</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" s="3"/>
+      <c r="D34" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="E34" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" s="3">
         <v>1</v>
       </c>
-      <c r="G34" s="5" t="s">
-        <v>105</v>
+      <c r="G34" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A35" s="3">
-        <v>101</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5" t="s">
-        <v>174</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
+        <v>41</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C35" s="3"/>
+      <c r="D35" s="14" t="s">
+        <v>199</v>
       </c>
       <c r="E35" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" s="3">
-        <v>3</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A36" s="3">
+        <v>2</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H35" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>64</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="3"/>
+      <c r="D36" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E36" s="3">
+        <v>2</v>
+      </c>
+      <c r="F36" s="3">
+        <v>1</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
         <v>73</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B37" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="E36" s="3">
-        <v>2</v>
-      </c>
-      <c r="F36" s="3">
-        <v>1</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="H36" s="10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A37" s="3">
-        <v>36</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="C37" s="5"/>
       <c r="D37" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E37" s="3">
         <v>2</v>
       </c>
       <c r="F37" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>113</v>
+        <v>71</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
       <c r="E38" s="3">
         <v>2</v>
       </c>
       <c r="F38" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>181</v>
+        <v>73</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
-        <v>38</v>
+        <v>83</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>115</v>
+        <v>75</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>116</v>
+        <v>76</v>
       </c>
       <c r="E39" s="3">
         <v>1</v>
@@ -1925,20 +1925,22 @@
         <v>1</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="H39" s="10"/>
-    </row>
-    <row r="40" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A40" s="3">
-        <v>8</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5" t="s">
-        <v>119</v>
+        <v>77</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A40" s="2">
+        <v>85</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C40" s="3"/>
+      <c r="D40" s="8" t="s">
+        <v>164</v>
       </c>
       <c r="E40" s="3">
         <v>1</v>
@@ -1946,232 +1948,233 @@
       <c r="F40" s="3">
         <v>1</v>
       </c>
-      <c r="G40" s="5" t="s">
-        <v>120</v>
+      <c r="G40" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A41" s="3">
-        <v>33</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="E41" s="7">
-        <v>1</v>
-      </c>
-      <c r="F41" s="7">
-        <v>1</v>
-      </c>
-      <c r="G41" s="5" t="s">
-        <v>123</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A41" s="2">
+        <v>85</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C41" s="3"/>
+      <c r="D41" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="E41" s="3">
+        <v>1</v>
+      </c>
+      <c r="F41" s="3">
+        <v>1</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>43</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="E42" s="7">
-        <v>1</v>
-      </c>
-      <c r="F42" s="7">
+        <v>84</v>
+      </c>
+      <c r="E42" s="3">
+        <v>2</v>
+      </c>
+      <c r="F42" s="3">
         <v>1</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>126</v>
+        <v>85</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="34" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>128</v>
+        <v>87</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="E43" s="7">
-        <v>1</v>
-      </c>
-      <c r="F43" s="7">
-        <v>1</v>
+        <v>88</v>
+      </c>
+      <c r="E43" s="3">
+        <v>2</v>
+      </c>
+      <c r="F43" s="3">
+        <v>3</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>131</v>
+        <v>90</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>185</v>
+        <v>91</v>
       </c>
       <c r="E44" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F44" s="3">
+        <v>2</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A45" s="2">
+        <v>93</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C45" s="3"/>
+      <c r="D45" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="E45" s="3">
+        <v>1</v>
+      </c>
+      <c r="F45" s="3">
+        <v>2</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A46" s="2">
+        <v>96</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" s="3"/>
+      <c r="D46" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E46" s="3">
+        <v>2</v>
+      </c>
+      <c r="F46" s="3">
+        <v>1</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H46" s="8" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>99</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E47" s="3">
+        <v>2</v>
+      </c>
+      <c r="F47" s="3">
+        <v>1</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>101</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E48" s="3">
+        <v>2</v>
+      </c>
+      <c r="F48" s="3">
+        <v>1</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H48" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>101</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E49" s="3">
+        <v>1</v>
+      </c>
+      <c r="F49" s="3">
         <v>3</v>
       </c>
-      <c r="G44" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="H44" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A45" s="3">
-        <v>36</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="E45" s="3">
-        <v>4</v>
-      </c>
-      <c r="F45" s="3">
-        <v>2</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A46" s="7">
-        <v>7</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E46" s="7">
-        <v>2</v>
-      </c>
-      <c r="F46" s="7">
-        <v>3</v>
-      </c>
-      <c r="G46" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="H46" s="10" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="51" x14ac:dyDescent="0.2">
-      <c r="A47">
-        <v>12</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="E47" s="7">
-        <v>2</v>
-      </c>
-      <c r="F47">
-        <v>2</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="H47" s="12" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="34" x14ac:dyDescent="0.2">
-      <c r="A48">
-        <v>15</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="E48">
-        <v>2</v>
-      </c>
-      <c r="F48">
-        <v>3</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>192</v>
-      </c>
-      <c r="H48" s="12" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A49">
-        <v>6</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="E49">
-        <v>4</v>
-      </c>
-      <c r="F49">
-        <v>4</v>
-      </c>
-      <c r="G49" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="H49" s="12" t="s">
-        <v>197</v>
+      <c r="G49" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I49">
+    <sortCondition ref="A1:A49"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>

</xml_diff>